<commit_message>
Settings sheet in questions.xlsx: defaults baked into every world
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to edit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to edit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questions'!$A$1:$L$153</definedName>
@@ -65,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -75,6 +76,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9955,6 +9957,642 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>What it does - these are the values EVERY new world starts with (rebuild after editing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Difficulty</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Normal or Hard</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Interval (minutes)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1 - 30, minutes between questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Score display</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>On or Off - the sidebar with next question / correct / wrong</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Menu on first join</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>On = the menu opens once per world when you join</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Rewards</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>On/Off</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Off = can never happen (you can still switch it in game, per world)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Classic tools</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Night Vision</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Slow Falling</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Safe spawn</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>+1 heart</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Full belly</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Second wind</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>64 Cobblestone</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Iron pickaxe</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Time freeze</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Useful item</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Bow + arrows</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fire Res 3 min</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Haste 3 min</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Speed 3 min</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Long arms</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tiny</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Punishments</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>On/Off</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Off = can never happen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Giant</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Short arms</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Glass bones</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Slowness II</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Mining Fatigue</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Levitation V</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Lost</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Mob wave</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Warden</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sky drop</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Wither</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Starvation</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Lights out</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Butterfingers</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Back to spawn</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Poison II</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Feeble</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Phantom night</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Creeper ambush</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Armor strip</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Tool break</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Buried alive</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B4:B5 B7:B50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"On,Off"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Normal,Hard"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9968,9 +10606,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -10013,9 +10649,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -10044,9 +10678,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>

</xml_diff>